<commit_message>
Updated locator for claimcreation
</commit_message>
<xml_diff>
--- a/tests/testdata/claimCenter/ClaimCenterData.xlsx
+++ b/tests/testdata/claimCenter/ClaimCenterData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Automation\playwrightclaimspoc\claimcenter-automation\tests\testdata\claimCenter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27AABF7F-4E2B-41A9-9FAE-51532578A05E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F22ECDC9-512B-42A0-A65C-84925FC59853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="38">
   <si>
     <t>TCID</t>
   </si>
@@ -115,6 +115,30 @@
   </si>
   <si>
     <t>Theft of entire vehicle</t>
+  </si>
+  <si>
+    <t>TC2</t>
+  </si>
+  <si>
+    <t>TC3</t>
+  </si>
+  <si>
+    <t>POL124</t>
+  </si>
+  <si>
+    <t>POL126</t>
+  </si>
+  <si>
+    <t>Jacob</t>
+  </si>
+  <si>
+    <t>Murphy</t>
+  </si>
+  <si>
+    <t>Keith</t>
+  </si>
+  <si>
+    <t>Rennon</t>
   </si>
 </sst>
 </file>
@@ -434,7 +458,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="12.90625" customWidth="1"/>
@@ -545,6 +569,100 @@
         <v>29</v>
       </c>
     </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Updated Data to multiple sheets
</commit_message>
<xml_diff>
--- a/tests/testdata/claimCenter/ClaimCenterData.xlsx
+++ b/tests/testdata/claimCenter/ClaimCenterData.xlsx
@@ -8,12 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Automation\playwrightclaimspoc\claimcenter-automation\tests\testdata\claimCenter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F22ECDC9-512B-42A0-A65C-84925FC59853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22805820-2F45-475D-B995-402346281B8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="claimsData" sheetId="1" r:id="rId1"/>
+    <sheet name="policyData" sheetId="2" r:id="rId1"/>
+    <sheet name="lossData" sheetId="3" r:id="rId2"/>
+    <sheet name="exposureData" sheetId="4" r:id="rId3"/>
+    <sheet name="reservesData" sheetId="5" r:id="rId4"/>
+    <sheet name="checkData" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="74">
   <si>
     <t>TCID</t>
   </si>
@@ -96,9 +100,6 @@
     <t>Mechanicsville</t>
   </si>
   <si>
-    <t>VA</t>
-  </si>
-  <si>
     <t>23116</t>
   </si>
   <si>
@@ -139,6 +140,117 @@
   </si>
   <si>
     <t>Rennon</t>
+  </si>
+  <si>
+    <t>lob</t>
+  </si>
+  <si>
+    <t>coverageType</t>
+  </si>
+  <si>
+    <t>coverageSubType</t>
+  </si>
+  <si>
+    <t>claimant</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>vehicleCondition</t>
+  </si>
+  <si>
+    <t>vehicleType</t>
+  </si>
+  <si>
+    <t>vehicleYear</t>
+  </si>
+  <si>
+    <t>vehicleMake</t>
+  </si>
+  <si>
+    <t>vehicleModel</t>
+  </si>
+  <si>
+    <t>vehicleStyle</t>
+  </si>
+  <si>
+    <t>vehicleColor</t>
+  </si>
+  <si>
+    <t>vehicleLicensePlate</t>
+  </si>
+  <si>
+    <t>vehicleLicenseState</t>
+  </si>
+  <si>
+    <t>vehicleVIN</t>
+  </si>
+  <si>
+    <t>vehicleStolen</t>
+  </si>
+  <si>
+    <t>vehicleParked</t>
+  </si>
+  <si>
+    <t>vehicleDamage</t>
+  </si>
+  <si>
+    <t>faultRating</t>
+  </si>
+  <si>
+    <t>vehicle</t>
+  </si>
+  <si>
+    <t>exposure</t>
+  </si>
+  <si>
+    <t>costType</t>
+  </si>
+  <si>
+    <t>costCategory</t>
+  </si>
+  <si>
+    <t>coverage</t>
+  </si>
+  <si>
+    <t>availableReserve</t>
+  </si>
+  <si>
+    <t>Vehicle</t>
+  </si>
+  <si>
+    <t>Claim Cost</t>
+  </si>
+  <si>
+    <t>Collision</t>
+  </si>
+  <si>
+    <t>Auto parts</t>
+  </si>
+  <si>
+    <t>200</t>
+  </si>
+  <si>
+    <t>John Doe</t>
+  </si>
+  <si>
+    <t>Insured</t>
+  </si>
+  <si>
+    <t>MV98989</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>Payee</t>
+  </si>
+  <si>
+    <t>Smith</t>
+  </si>
+  <si>
+    <t>Virginia</t>
   </si>
 </sst>
 </file>
@@ -457,214 +569,465 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABB5CCD5-1F8C-4E91-9FFB-EFFF5DA356DA}">
+  <dimension ref="A1:N4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="12.90625" customWidth="1"/>
-    <col min="3" max="3" width="11.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.6328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.08984375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.6328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.90625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="23.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.36328125" customWidth="1"/>
+    <col min="3" max="3" width="14.7265625" customWidth="1"/>
+    <col min="4" max="4" width="12.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="N1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="L2" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="M2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="N2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="M2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="O2" s="1" t="s">
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>30</v>
       </c>
       <c r="B3" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D3" s="2" t="s">
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="H3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H3" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="I3" s="2" t="s">
+      <c r="J3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="K3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="L3" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="M3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="N3" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="M3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="O3" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" s="2" t="s">
+      <c r="I4" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="H4" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="I4" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="L4" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="M4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="N4" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="O4" s="1" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04AC9C0C-3AE5-4A61-B383-305FB5E68ACA}">
+  <dimension ref="A1:Q4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="16.453125" customWidth="1"/>
+    <col min="3" max="3" width="21.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I1" t="s">
+        <v>47</v>
+      </c>
+      <c r="J1" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1" t="s">
+        <v>49</v>
+      </c>
+      <c r="L1" t="s">
+        <v>50</v>
+      </c>
+      <c r="M1" t="s">
+        <v>51</v>
+      </c>
+      <c r="N1" t="s">
+        <v>52</v>
+      </c>
+      <c r="O1" t="s">
+        <v>53</v>
+      </c>
+      <c r="P1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5555805B-3114-4A15-8ACE-E2F5F885514D}">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="12.36328125" customWidth="1"/>
+    <col min="3" max="4" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F2" t="s">
+        <v>68</v>
+      </c>
+      <c r="G2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE23A9C7-4C45-42B9-B210-82302D40347F}">
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="10.1796875" customWidth="1"/>
+    <col min="3" max="3" width="9.54296875" customWidth="1"/>
+    <col min="4" max="4" width="9.6328125" customWidth="1"/>
+    <col min="5" max="5" width="13.90625" customWidth="1"/>
+    <col min="6" max="6" width="18.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{612423C4-94FD-4B38-AA42-104AE678E3C8}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>300</v>
+      </c>
+      <c r="C2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added 3 LOB data
</commit_message>
<xml_diff>
--- a/tests/testdata/claimCenter/ClaimCenterData.xlsx
+++ b/tests/testdata/claimCenter/ClaimCenterData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Automation\playwrightclaimspoc\claimcenter-automation\tests\testdata\claimCenter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22805820-2F45-475D-B995-402346281B8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71E462FA-D416-482C-B566-F3909F329BE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="policyData" sheetId="2" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="77">
   <si>
     <t>TCID</t>
   </si>
@@ -251,6 +251,15 @@
   </si>
   <si>
     <t>Virginia</t>
+  </si>
+  <si>
+    <t>Commercial Auto</t>
+  </si>
+  <si>
+    <t>Homeowners</t>
+  </si>
+  <si>
+    <t>Hail</t>
   </si>
 </sst>
 </file>
@@ -671,10 +680,10 @@
         <v>29</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>74</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>74</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>31</v>
@@ -715,10 +724,10 @@
         <v>30</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>75</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>75</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>32</v>
@@ -851,7 +860,7 @@
         <v>27</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>28</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -911,6 +920,18 @@
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>29</v>
+      </c>
+      <c r="D3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E3" t="s">
+        <v>67</v>
+      </c>
+      <c r="F3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G3" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">

</xml_diff>